<commit_message>
FEAT: validation of output
</commit_message>
<xml_diff>
--- a/templates/AARR_Modelo de datos_template.xlsx
+++ b/templates/AARR_Modelo de datos_template.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Workspaces\OCR_tests - uv\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77173ACD-3867-4DB7-933D-3238A1F2B59E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A4FB8D1-EFC8-4FA7-A1EC-A9948C9777FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{5BEF5658-777B-40B8-A208-7E392796F3C3}"/>
   </bookViews>
   <sheets>
     <sheet name="AARR" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191028"/>
+  <calcPr calcId="191028" calcOnSave="0"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="48">
   <si>
     <t>Orígenes de datos</t>
   </si>
@@ -134,21 +134,12 @@
     <t>Detalle/Justifiación</t>
   </si>
   <si>
-    <t>¿Es este tratamiento similar a otro para el que haya sido necesario realizar un</t>
-  </si>
-  <si>
     <t>Detalle/Justificacación</t>
   </si>
   <si>
-    <t>¿Este tratamiento puede conllevar una pérdida o alteración de la información</t>
-  </si>
-  <si>
     <t>Justificación</t>
   </si>
   <si>
-    <t>¿Se utilizada documentación en papel para tratar datos personales?</t>
-  </si>
-  <si>
     <t>¿Interviene algún proveedor en el proceso?</t>
   </si>
   <si>
@@ -161,7 +152,34 @@
     <t>¿Se prevén efectos colaterales o adversos para los interesados?</t>
   </si>
   <si>
-    <t>Resultado del análisis</t>
+    <t>¿Es este tratamiento similar a otro para el que haya sido necesario realizar un EIPD?</t>
+  </si>
+  <si>
+    <t>¿Este tratamiento puede conllevar una pérdida o alteración de la información?</t>
+  </si>
+  <si>
+    <t>¿Es utilizada documentación en papel para tratar datos personales?</t>
+  </si>
+  <si>
+    <t>¿En base a las respuestas realizadas en el cuestionario de evaluación objetiva, debe calificarse la presente actividad de tratamiento como de "RIESGO ALTO" para los derechos y libertades de las personas?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ha indicado que la presente actividad presenta riesgo ESCASO o NULO, por lo tanto no existe la obligación de realizar un PIA. Por favor, indique los motivos que justifican esta decisión como resultado del análisis </t>
+  </si>
+  <si>
+    <t>Evidencias relativas al resultado del análisis: con riesgo ESCASO o NULO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ha indicado que la presente actividad presenta RIESGO ALTO, por lo tanto existe la obligación de realizar un PIA. Por favor, indique los motivos que justifican esta decisión como resultado del análisis </t>
+  </si>
+  <si>
+    <t>Evidencias relativas al resultado del análisis: RIESGO ALTO</t>
+  </si>
+  <si>
+    <t>Otra información relevante de procedimientos anteriores</t>
+  </si>
+  <si>
+    <t>Evidencias de otro tipo de información relevante adicional</t>
   </si>
 </sst>
 </file>
@@ -787,46 +805,64 @@
         <v>31</v>
       </c>
       <c r="AR2" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="AS2" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="AS2" s="2" t="s">
+      <c r="AT2" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="AU2" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="AT2" s="2" t="s">
+      <c r="AV2" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="AW2" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="AX2" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="AU2" s="2" t="s">
+      <c r="AY2" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="AZ2" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="AV2" s="2" t="s">
+      <c r="BA2" s="2" t="s">
         <v>36</v>
-      </c>
-      <c r="AW2" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="AX2" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="AY2" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="AZ2" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="BA2" s="2" t="s">
-        <v>39</v>
       </c>
       <c r="BB2" s="2" t="s">
         <v>23</v>
       </c>
       <c r="BC2" s="2" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="BD2" s="2" t="s">
         <v>23</v>
       </c>
       <c r="BE2" s="2" t="s">
         <v>41</v>
+      </c>
+      <c r="BF2" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="BG2" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="BH2" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="BI2" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="BJ2" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="BK2" s="2" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="9" spans="2:107" x14ac:dyDescent="0.3">
@@ -840,12 +876,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101000148212AB4668C49858BD42EF6132060" ma:contentTypeVersion="3" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="713bb1124bf86e0d5d9ff0ef7b1b0168">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="05e1840a-b6a9-40a5-8391-9518f72c2bda" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="07d428b5caee6bae41599bc558c95588" ns2:_="">
     <xsd:import namespace="05e1840a-b6a9-40a5-8391-9518f72c2bda"/>
@@ -983,6 +1013,12 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -993,15 +1029,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C443E8A2-E353-40BE-B576-7371C1BF9C59}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CE34A8AB-C0F5-42C0-9770-06CB9201723D}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1019,6 +1046,15 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C443E8A2-E353-40BE-B576-7371C1BF9C59}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E28DF92D-FB35-4D5B-B297-C807C06B1307}">
   <ds:schemaRefs>

</xml_diff>

<commit_message>
ajustes finales modelo AARR html
</commit_message>
<xml_diff>
--- a/templates/AARR_Modelo de datos_template.xlsx
+++ b/templates/AARR_Modelo de datos_template.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Workspaces\OCR_tests - uv\templates\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\.git\asisa_ocr\asisaocr\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A4FB8D1-EFC8-4FA7-A1EC-A9948C9777FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84CB0169-4179-424E-9DA9-ECC8607B782B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{5BEF5658-777B-40B8-A208-7E392796F3C3}"/>
+    <workbookView xWindow="-108" yWindow="-13068" windowWidth="23256" windowHeight="13176" xr2:uid="{5BEF5658-777B-40B8-A208-7E392796F3C3}"/>
   </bookViews>
   <sheets>
     <sheet name="AARR" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191028" calcOnSave="0"/>
+  <calcPr calcId="191028"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="50">
   <si>
     <t>Orígenes de datos</t>
   </si>
@@ -80,9 +80,6 @@
     <t>¿El tratamiento de los datos implica una toma de decisiones automatizada sin que haya ninguna persona que intervenga en la decisión o valore los resultados?</t>
   </si>
   <si>
-    <t>Detalle/Justificación (si existe)</t>
-  </si>
-  <si>
     <t>La recogida de los datos tiene como finalidad la monitorización o evaluación sistemática y exhaustiva de aspectos personales?</t>
   </si>
   <si>
@@ -107,9 +104,6 @@
     <t>¿Se enriquece la información de los interesados mediante la recogida de nuevas categorías de datos o se usen las existentes con nuevas finalidades que antes no se contemplaban, en particular, si estas finalidades son más intrusivas o inesperadas para los afectados, o incluso pueda llegar a bloquear el disfrute de algún servicio?</t>
   </si>
   <si>
-    <t>Detalle/justificación</t>
-  </si>
-  <si>
     <t>¿El tratamiento implica que un elevado número de personas (más allá de las necesarias para llevar a cabo el mismo) tenga acceso a los datos personales tratados?</t>
   </si>
   <si>
@@ -131,15 +125,6 @@
     <t>¿Se realizan transferencias internacionales de datos a países fuera de la Unión Europea y que no cuenten con medidas de protección de datos de carácter personal similares a las establecidas por la Autoridad de Control ?</t>
   </si>
   <si>
-    <t>Detalle/Justifiación</t>
-  </si>
-  <si>
-    <t>Detalle/Justificacación</t>
-  </si>
-  <si>
-    <t>Justificación</t>
-  </si>
-  <si>
     <t>¿Interviene algún proveedor en el proceso?</t>
   </si>
   <si>
@@ -180,6 +165,27 @@
   </si>
   <si>
     <t>Evidencias de otro tipo de información relevante adicional</t>
+  </si>
+  <si>
+    <t>Indique los sistemas en los que se tratarán los datos (Medios electrónicos (físicos o en la nube)/Papel)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">¿Existen fines secundarios/intermedios con el tratamiento de los datos? </t>
+  </si>
+  <si>
+    <t>Especificar cuáles son los fines secundarios/intermedios</t>
+  </si>
+  <si>
+    <t>¿Con qué frecuencia se recaban los datos?</t>
+  </si>
+  <si>
+    <t>¿Se recaban todos los datos afectados de forma conjunta o en distintos momentos?</t>
+  </si>
+  <si>
+    <t>Descripción del ciclo de vida</t>
+  </si>
+  <si>
+    <t>Tratamiento / Finalidad</t>
   </si>
 </sst>
 </file>
@@ -222,12 +228,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -510,126 +519,120 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B5714997-6257-4473-9DF2-1584408E574C}">
-  <dimension ref="B1:DC9"/>
+  <dimension ref="B1:DJ9"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="17.33203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="11.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="25.88671875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="35.5546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="53.6640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="83.33203125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="55.21875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="140.5546875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="169.33203125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="83.6640625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="55.77734375" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="24.6640625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="69" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="15.6640625" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="23.88671875" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="32.21875" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="50.77734375" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="50.44140625" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="69.6640625" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="106.6640625" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="13.109375" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="163.88671875" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="13.109375" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="132" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="13.109375" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="134.109375" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="13.109375" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="116.6640625" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="13.109375" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="9.88671875" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="87.77734375" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="50.21875" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="63.21875" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="123.5546875" bestFit="1" customWidth="1"/>
-    <col min="35" max="35" width="36.77734375" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="31.88671875" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="44.44140625" bestFit="1" customWidth="1"/>
-    <col min="38" max="38" width="51.5546875" bestFit="1" customWidth="1"/>
-    <col min="39" max="39" width="46.5546875" bestFit="1" customWidth="1"/>
-    <col min="40" max="40" width="99.21875" bestFit="1" customWidth="1"/>
-    <col min="41" max="41" width="24.88671875" bestFit="1" customWidth="1"/>
-    <col min="42" max="42" width="55.21875" bestFit="1" customWidth="1"/>
-    <col min="43" max="43" width="66.6640625" bestFit="1" customWidth="1"/>
-    <col min="44" max="44" width="23" bestFit="1" customWidth="1"/>
-    <col min="45" max="45" width="49.77734375" bestFit="1" customWidth="1"/>
-    <col min="46" max="46" width="24.77734375" bestFit="1" customWidth="1"/>
-    <col min="47" max="47" width="34.21875" bestFit="1" customWidth="1"/>
-    <col min="48" max="48" width="26" bestFit="1" customWidth="1"/>
-    <col min="49" max="49" width="32.44140625" bestFit="1" customWidth="1"/>
-    <col min="50" max="50" width="30.77734375" bestFit="1" customWidth="1"/>
-    <col min="51" max="51" width="33.88671875" bestFit="1" customWidth="1"/>
-    <col min="52" max="52" width="26" bestFit="1" customWidth="1"/>
-    <col min="53" max="53" width="25.77734375" bestFit="1" customWidth="1"/>
-    <col min="54" max="54" width="30.21875" bestFit="1" customWidth="1"/>
-    <col min="55" max="55" width="11.33203125" bestFit="1" customWidth="1"/>
-    <col min="56" max="56" width="25.88671875" bestFit="1" customWidth="1"/>
-    <col min="57" max="57" width="35.5546875" bestFit="1" customWidth="1"/>
-    <col min="58" max="58" width="53.6640625" bestFit="1" customWidth="1"/>
-    <col min="59" max="59" width="83.33203125" bestFit="1" customWidth="1"/>
-    <col min="60" max="60" width="55.21875" bestFit="1" customWidth="1"/>
-    <col min="61" max="61" width="140.5546875" bestFit="1" customWidth="1"/>
-    <col min="62" max="62" width="169.33203125" bestFit="1" customWidth="1"/>
-    <col min="63" max="63" width="83.6640625" bestFit="1" customWidth="1"/>
-    <col min="64" max="64" width="55.77734375" bestFit="1" customWidth="1"/>
-    <col min="65" max="65" width="24.6640625" bestFit="1" customWidth="1"/>
-    <col min="66" max="66" width="69" bestFit="1" customWidth="1"/>
-    <col min="67" max="67" width="15.6640625" bestFit="1" customWidth="1"/>
-    <col min="68" max="68" width="23.88671875" bestFit="1" customWidth="1"/>
-    <col min="69" max="69" width="32.21875" bestFit="1" customWidth="1"/>
-    <col min="70" max="70" width="50.77734375" bestFit="1" customWidth="1"/>
-    <col min="71" max="71" width="50.44140625" bestFit="1" customWidth="1"/>
-    <col min="72" max="72" width="69.6640625" bestFit="1" customWidth="1"/>
-    <col min="73" max="73" width="106.6640625" bestFit="1" customWidth="1"/>
-    <col min="74" max="74" width="13.109375" bestFit="1" customWidth="1"/>
-    <col min="75" max="75" width="163.88671875" bestFit="1" customWidth="1"/>
-    <col min="76" max="76" width="13.109375" bestFit="1" customWidth="1"/>
-    <col min="77" max="77" width="132" bestFit="1" customWidth="1"/>
-    <col min="78" max="78" width="13.109375" bestFit="1" customWidth="1"/>
-    <col min="79" max="79" width="134.109375" bestFit="1" customWidth="1"/>
-    <col min="80" max="80" width="13.109375" bestFit="1" customWidth="1"/>
-    <col min="81" max="81" width="116.6640625" bestFit="1" customWidth="1"/>
-    <col min="82" max="82" width="13.109375" bestFit="1" customWidth="1"/>
-    <col min="83" max="83" width="9.88671875" bestFit="1" customWidth="1"/>
-    <col min="84" max="84" width="87.77734375" bestFit="1" customWidth="1"/>
-    <col min="85" max="85" width="50.21875" bestFit="1" customWidth="1"/>
-    <col min="86" max="86" width="63.21875" bestFit="1" customWidth="1"/>
-    <col min="87" max="87" width="123.5546875" bestFit="1" customWidth="1"/>
-    <col min="88" max="88" width="36.77734375" bestFit="1" customWidth="1"/>
-    <col min="89" max="89" width="31.88671875" bestFit="1" customWidth="1"/>
-    <col min="90" max="90" width="44.44140625" bestFit="1" customWidth="1"/>
-    <col min="91" max="91" width="51.5546875" bestFit="1" customWidth="1"/>
-    <col min="92" max="92" width="46.5546875" bestFit="1" customWidth="1"/>
-    <col min="93" max="93" width="99.21875" bestFit="1" customWidth="1"/>
-    <col min="94" max="94" width="24.88671875" bestFit="1" customWidth="1"/>
-    <col min="95" max="95" width="55.21875" bestFit="1" customWidth="1"/>
-    <col min="96" max="96" width="66.6640625" bestFit="1" customWidth="1"/>
-    <col min="97" max="97" width="23" bestFit="1" customWidth="1"/>
-    <col min="98" max="98" width="49.77734375" bestFit="1" customWidth="1"/>
-    <col min="99" max="99" width="24.77734375" bestFit="1" customWidth="1"/>
-    <col min="100" max="100" width="34.21875" bestFit="1" customWidth="1"/>
-    <col min="101" max="101" width="26" bestFit="1" customWidth="1"/>
-    <col min="102" max="102" width="32.44140625" bestFit="1" customWidth="1"/>
-    <col min="103" max="103" width="30.77734375" bestFit="1" customWidth="1"/>
-    <col min="104" max="104" width="33.88671875" bestFit="1" customWidth="1"/>
-    <col min="105" max="105" width="26" bestFit="1" customWidth="1"/>
-    <col min="106" max="106" width="25.77734375" bestFit="1" customWidth="1"/>
-    <col min="107" max="108" width="30.21875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.77734375" customWidth="1"/>
+    <col min="3" max="3" width="11.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="25.88671875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="35.5546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="53.6640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="83.33203125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="55.21875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="140.5546875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="169.33203125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="83.6640625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="55.77734375" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="24.6640625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="69" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="15.6640625" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="23.88671875" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="32.21875" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="50.77734375" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="50.44140625" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="69.6640625" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="106.6640625" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="13.109375" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="163.88671875" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="13.109375" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="132" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="13.109375" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="134.109375" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="13.109375" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="116.6640625" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="13.109375" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="9.88671875" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="87.77734375" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="50.21875" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="63.21875" bestFit="1" customWidth="1"/>
+    <col min="35" max="35" width="123.5546875" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="36.77734375" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="31.88671875" bestFit="1" customWidth="1"/>
+    <col min="38" max="38" width="44.44140625" bestFit="1" customWidth="1"/>
+    <col min="39" max="39" width="51.5546875" bestFit="1" customWidth="1"/>
+    <col min="40" max="40" width="46.5546875" bestFit="1" customWidth="1"/>
+    <col min="41" max="41" width="99.21875" bestFit="1" customWidth="1"/>
+    <col min="42" max="42" width="24.88671875" bestFit="1" customWidth="1"/>
+    <col min="43" max="43" width="55.21875" bestFit="1" customWidth="1"/>
+    <col min="44" max="44" width="66.6640625" bestFit="1" customWidth="1"/>
+    <col min="45" max="45" width="23" bestFit="1" customWidth="1"/>
+    <col min="46" max="46" width="49.77734375" bestFit="1" customWidth="1"/>
+    <col min="47" max="47" width="24.77734375" bestFit="1" customWidth="1"/>
+    <col min="48" max="48" width="34.21875" bestFit="1" customWidth="1"/>
+    <col min="49" max="49" width="26" bestFit="1" customWidth="1"/>
+    <col min="50" max="50" width="32.44140625" bestFit="1" customWidth="1"/>
+    <col min="51" max="51" width="30.77734375" bestFit="1" customWidth="1"/>
+    <col min="52" max="52" width="33.88671875" bestFit="1" customWidth="1"/>
+    <col min="53" max="58" width="33.88671875" customWidth="1"/>
+    <col min="59" max="59" width="26" bestFit="1" customWidth="1"/>
+    <col min="60" max="60" width="25.77734375" bestFit="1" customWidth="1"/>
+    <col min="61" max="61" width="30.21875" bestFit="1" customWidth="1"/>
+    <col min="62" max="62" width="11.33203125" bestFit="1" customWidth="1"/>
+    <col min="63" max="63" width="25.88671875" bestFit="1" customWidth="1"/>
+    <col min="64" max="64" width="35.5546875" bestFit="1" customWidth="1"/>
+    <col min="65" max="65" width="53.6640625" bestFit="1" customWidth="1"/>
+    <col min="66" max="66" width="83.33203125" bestFit="1" customWidth="1"/>
+    <col min="67" max="67" width="55.21875" bestFit="1" customWidth="1"/>
+    <col min="68" max="68" width="140.5546875" bestFit="1" customWidth="1"/>
+    <col min="69" max="69" width="169.33203125" bestFit="1" customWidth="1"/>
+    <col min="70" max="70" width="83.6640625" bestFit="1" customWidth="1"/>
+    <col min="71" max="71" width="55.77734375" bestFit="1" customWidth="1"/>
+    <col min="72" max="72" width="24.6640625" bestFit="1" customWidth="1"/>
+    <col min="73" max="73" width="69" bestFit="1" customWidth="1"/>
+    <col min="74" max="74" width="15.6640625" bestFit="1" customWidth="1"/>
+    <col min="75" max="75" width="23.88671875" bestFit="1" customWidth="1"/>
+    <col min="76" max="76" width="32.21875" bestFit="1" customWidth="1"/>
+    <col min="77" max="77" width="50.77734375" bestFit="1" customWidth="1"/>
+    <col min="78" max="78" width="50.44140625" bestFit="1" customWidth="1"/>
+    <col min="79" max="79" width="69.6640625" bestFit="1" customWidth="1"/>
+    <col min="80" max="80" width="106.6640625" bestFit="1" customWidth="1"/>
+    <col min="81" max="81" width="13.109375" bestFit="1" customWidth="1"/>
+    <col min="82" max="82" width="163.88671875" bestFit="1" customWidth="1"/>
+    <col min="83" max="83" width="13.109375" bestFit="1" customWidth="1"/>
+    <col min="84" max="84" width="132" bestFit="1" customWidth="1"/>
+    <col min="85" max="85" width="13.109375" bestFit="1" customWidth="1"/>
+    <col min="86" max="86" width="134.109375" bestFit="1" customWidth="1"/>
+    <col min="87" max="87" width="13.109375" bestFit="1" customWidth="1"/>
+    <col min="88" max="88" width="116.6640625" bestFit="1" customWidth="1"/>
+    <col min="89" max="89" width="13.109375" bestFit="1" customWidth="1"/>
+    <col min="90" max="90" width="9.88671875" bestFit="1" customWidth="1"/>
+    <col min="91" max="91" width="87.77734375" bestFit="1" customWidth="1"/>
+    <col min="92" max="92" width="50.21875" bestFit="1" customWidth="1"/>
+    <col min="93" max="93" width="63.21875" bestFit="1" customWidth="1"/>
+    <col min="94" max="94" width="123.5546875" bestFit="1" customWidth="1"/>
+    <col min="95" max="95" width="36.77734375" bestFit="1" customWidth="1"/>
+    <col min="96" max="96" width="31.88671875" bestFit="1" customWidth="1"/>
+    <col min="97" max="97" width="44.44140625" bestFit="1" customWidth="1"/>
+    <col min="98" max="98" width="51.5546875" bestFit="1" customWidth="1"/>
+    <col min="99" max="99" width="46.5546875" bestFit="1" customWidth="1"/>
+    <col min="100" max="100" width="99.21875" bestFit="1" customWidth="1"/>
+    <col min="101" max="101" width="24.88671875" bestFit="1" customWidth="1"/>
+    <col min="102" max="102" width="55.21875" bestFit="1" customWidth="1"/>
+    <col min="103" max="103" width="66.6640625" bestFit="1" customWidth="1"/>
+    <col min="104" max="104" width="23" bestFit="1" customWidth="1"/>
+    <col min="105" max="105" width="49.77734375" bestFit="1" customWidth="1"/>
+    <col min="106" max="106" width="24.77734375" bestFit="1" customWidth="1"/>
+    <col min="107" max="107" width="34.21875" bestFit="1" customWidth="1"/>
+    <col min="108" max="108" width="26" bestFit="1" customWidth="1"/>
+    <col min="109" max="109" width="32.44140625" bestFit="1" customWidth="1"/>
+    <col min="110" max="110" width="30.77734375" bestFit="1" customWidth="1"/>
+    <col min="111" max="111" width="33.88671875" bestFit="1" customWidth="1"/>
+    <col min="112" max="112" width="26" bestFit="1" customWidth="1"/>
+    <col min="113" max="113" width="25.77734375" bestFit="1" customWidth="1"/>
+    <col min="114" max="115" width="30.21875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:107" x14ac:dyDescent="0.3">
-      <c r="BC1" s="1"/>
-      <c r="BD1" s="1"/>
-      <c r="BE1" s="1"/>
-      <c r="BF1" s="1"/>
-      <c r="BG1" s="1"/>
-      <c r="BH1" s="1"/>
-      <c r="BI1" s="1"/>
+    <row r="1" spans="2:114" x14ac:dyDescent="0.3">
       <c r="BJ1" s="1"/>
       <c r="BK1" s="1"/>
       <c r="BL1" s="1"/>
@@ -676,206 +679,244 @@
       <c r="DA1" s="1"/>
       <c r="DB1" s="1"/>
       <c r="DC1" s="1"/>
+      <c r="DD1" s="1"/>
+      <c r="DE1" s="1"/>
+      <c r="DF1" s="1"/>
+      <c r="DG1" s="1"/>
+      <c r="DH1" s="1"/>
+      <c r="DI1" s="1"/>
+      <c r="DJ1" s="1"/>
     </row>
-    <row r="2" spans="2:107" ht="328.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="2" t="s">
+    <row r="2" spans="2:114" ht="100.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B2" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="C2" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="D2" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="E2" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="F2" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="G2" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="G2" s="2" t="s">
+      <c r="H2" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="H2" s="2" t="s">
+      <c r="I2" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="I2" s="2" t="s">
+      <c r="J2" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="J2" s="2" t="s">
+      <c r="K2" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="K2" s="2" t="s">
+      <c r="L2" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="L2" s="2" t="s">
+      <c r="M2" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="M2" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="N2" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="O2" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="O2" s="2" t="s">
+      <c r="P2" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="Q2" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="P2" s="2" t="s">
+      <c r="R2" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="S2" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="Q2" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="R2" s="2" t="s">
+      <c r="T2" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="U2" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="S2" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="T2" s="2" t="s">
+      <c r="V2" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="W2" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="U2" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="V2" s="2" t="s">
+      <c r="X2" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="Y2" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="W2" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="X2" s="2" t="s">
+      <c r="Z2" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="AA2" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="Y2" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="Z2" s="2" t="s">
+      <c r="AB2" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="AC2" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="AA2" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="AB2" s="2" t="s">
+      <c r="AD2" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="AE2" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="AC2" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="AD2" s="2" t="s">
+      <c r="AF2" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="AG2" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="AE2" s="2" t="s">
+      <c r="AH2" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="AI2" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="AF2" s="2" t="s">
+      <c r="AJ2" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="AK2" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="AG2" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="AH2" s="2" t="s">
+      <c r="AL2" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="AM2" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="AI2" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="AJ2" s="2" t="s">
+      <c r="AN2" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="AO2" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="AK2" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="AL2" s="2" t="s">
+      <c r="AP2" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="AM2" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="AN2" s="2" t="s">
+      <c r="AQ2" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="AO2" s="2" t="s">
+      <c r="AR2" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="AS2" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="AT2" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="AU2" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="AV2" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="AW2" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="AX2" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="AY2" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="AP2" s="2" t="s">
+      <c r="AZ2" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="BA2" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="BB2" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="BC2" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="BD2" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="BE2" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="BF2" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="BG2" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="AQ2" s="2" t="s">
+      <c r="BH2" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="AR2" s="2" t="s">
+      <c r="BI2" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="BJ2" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="BK2" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="BL2" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="BM2" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="BN2" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="AS2" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="AT2" s="2" t="s">
+      <c r="BO2" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="AU2" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="AV2" s="2" t="s">
+      <c r="BP2" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="AW2" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="AX2" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="AY2" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="AZ2" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="BA2" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="BB2" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="BC2" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="BD2" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="BE2" s="2" t="s">
+      <c r="BQ2" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="BF2" s="2" t="s">
+      <c r="BR2" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="BG2" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="BH2" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="BI2" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="BJ2" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="BK2" s="2" t="s">
-        <v>47</v>
-      </c>
     </row>
-    <row r="9" spans="2:107" x14ac:dyDescent="0.3">
-      <c r="M9" t="s">
+    <row r="9" spans="2:114" x14ac:dyDescent="0.3">
+      <c r="N9" t="s">
         <v>1</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101000148212AB4668C49858BD42EF6132060" ma:contentTypeVersion="3" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="713bb1124bf86e0d5d9ff0ef7b1b0168">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="05e1840a-b6a9-40a5-8391-9518f72c2bda" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="07d428b5caee6bae41599bc558c95588" ns2:_="">
     <xsd:import namespace="05e1840a-b6a9-40a5-8391-9518f72c2bda"/>
@@ -1013,22 +1054,21 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement/>
 </p:properties>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E28DF92D-FB35-4D5B-B297-C807C06B1307}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CE34A8AB-C0F5-42C0-9770-06CB9201723D}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1046,19 +1086,11 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C443E8A2-E353-40BE-B576-7371C1BF9C59}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E28DF92D-FB35-4D5B-B297-C807C06B1307}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>